<commit_message>
Strip em dashes and de-slop copy across README, dashboard, and Excel
Removes the top AI-writing tell (em dashes) everywhere, replaces two patterned
subheads (rule-of-three, antithesis) with plain descriptive lines, and fixes the
resulting punctuation. No numbers changed.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Houlihan Lokey - Financial Model.xlsx
+++ b/Houlihan Lokey - Financial Model.xlsx
@@ -581,14 +581,14 @@
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Segment revenue sums to total revenue — every fiscal year.</t>
+          <t xml:space="preserve">   • Segment revenue sums to total revenue, every fiscal year.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Quarterly revenue sums to the reported 10-K annual — every fiscal year.</t>
+          <t xml:space="preserve">   • Quarterly revenue sums to the reported 10-K annual, every fiscal year.</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Operating Model  —  $ in millions unless noted</t>
+          <t>Operating Model: $ in millions unless noted</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Quarterly Detail  —  the audit trail (annual columns above sum these)</t>
+          <t>Quarterly Detail: the audit trail (annual columns above sum these)</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Corporate Finance — closed transactions</t>
+          <t>Corporate Finance, closed transactions</t>
         </is>
       </c>
       <c r="C16" s="13" t="n">
@@ -1934,7 +1934,7 @@
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Financial Restructuring — closed transactions</t>
+          <t>Financial Restructuring, closed transactions</t>
         </is>
       </c>
       <c r="C17" s="13" t="n">

</xml_diff>